<commit_message>
Implement the excel importer.
Support to load excel file directly into UE as a curvetable.
</commit_message>
<xml_diff>
--- a/Document/CharacterTable.xlsx
+++ b/Document/CharacterTable.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>ID</t>
   </si>
@@ -29,12 +29,15 @@
   <si>
     <t>Icon</t>
   </si>
+  <si>
+    <t>CharacterTable</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -42,13 +45,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -63,8 +80,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -345,21 +366,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C2" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>